<commit_message>
Lite Pant: XS 15,2%; +1,6 pp L; resto de XS entre S y M
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LITE_PANT_RANGO_PRODUCCION.xlsx
+++ b/LITE_PANT_RANGO_PRODUCCION.xlsx
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1.5485</v>
+        <v>1.5523</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>mín · máx 785 und</t>
+          <t>mín · máx 783 und</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>mín · máx 298 und</t>
+          <t>mín · máx 297 und</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1288,24 +1288,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>L 16.6%</t>
+          <t>L 18.2%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>XS objetivo 18%</t>
+          <t>XS objetivo 15.2%</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>XS 18.0%</t>
+          <t>XS 15.2%</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Exceso repartido 50/50 a S y M · L/XL sin cambio</t>
+          <t>+1.6 pp a L · resto 50/50 S y M</t>
         </is>
       </c>
     </row>
@@ -1563,14 +1563,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>18.0%</t>
+          <t>15.2%</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
+        <v>138</v>
+      </c>
+      <c r="D5" s="8" t="n">
         <v>164</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>195</v>
       </c>
     </row>
     <row r="6">
@@ -1581,14 +1581,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>25.5%</t>
+          <t>26.1%</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7">
@@ -1599,14 +1599,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>29.1%</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8">
@@ -1617,14 +1617,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>16.6%</t>
+          <t>18.2%</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>180</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9">
@@ -1652,10 +1652,10 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
   </sheetData>
@@ -1699,14 +1699,14 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>Rango producción: 912 – 1083 und</t>
+          <t>Rango producción: 910 – 1080 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>MÍNIMO — 912 und (compromiso)</t>
+          <t>MÍNIMO — 910 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1754,22 +1754,22 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>77</v>
       </c>
       <c r="G7" s="17" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="8">
@@ -1779,19 +1779,19 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G8" s="17" t="n">
         <v>229</v>
@@ -1804,28 +1804,28 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>164</v>
+        <v>139</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>MÁXIMO — 1083 und (techo)</t>
+          <t>MÁXIMO — 1080 und (techo)</t>
         </is>
       </c>
     </row>
@@ -1873,22 +1873,22 @@
         </is>
       </c>
       <c r="B13" s="17" t="n">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D13" s="17" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E13" s="17" t="n">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>89</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="14">
@@ -1898,22 +1898,22 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="E14" s="17" t="n">
         <v>54</v>
       </c>
-      <c r="C14" s="17" t="n">
-        <v>76</v>
-      </c>
-      <c r="D14" s="17" t="n">
-        <v>85</v>
-      </c>
-      <c r="E14" s="17" t="n">
-        <v>50</v>
-      </c>
       <c r="F14" s="17" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15">
@@ -1923,22 +1923,22 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>195</v>
+        <v>164</v>
       </c>
       <c r="C15" s="19" t="n">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="17">
@@ -1982,10 +1982,10 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>1057.61</v>
+        <v>1057.02</v>
       </c>
       <c r="C19" s="23" t="n">
-        <v>1215.64</v>
+        <v>1215.54</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2005,10 +2005,10 @@
         </is>
       </c>
       <c r="B20" s="22" t="n">
-        <v>354.75</v>
+        <v>355.37</v>
       </c>
       <c r="C20" s="23" t="n">
-        <v>461.36</v>
+        <v>461.03</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2028,10 +2028,10 @@
         </is>
       </c>
       <c r="B21" s="22" t="n">
-        <v>1412.36</v>
+        <v>1412.39</v>
       </c>
       <c r="C21" s="23" t="n">
-        <v>1677</v>
+        <v>1676.57</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2051,10 +2051,10 @@
         </is>
       </c>
       <c r="B22" s="22" t="n">
-        <v>651.16</v>
+        <v>651.29</v>
       </c>
       <c r="C22" s="23" t="n">
-        <v>773.28</v>
+        <v>773</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2074,10 +2074,10 @@
         </is>
       </c>
       <c r="B23" s="22" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="C23" s="23" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2141,14 +2141,14 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 912 – 1083 und</t>
+          <t>Rango global: 910 – 1080 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
         <is>
-          <t>Negro (785 und máx)</t>
+          <t>Negro (783 und máx)</t>
         </is>
       </c>
     </row>
@@ -2243,28 +2243,28 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>77</v>
@@ -2280,16 +2280,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>Verde Militar (298 und máx)</t>
+          <t>Verde Militar (297 und máx)</t>
         </is>
       </c>
     </row>
@@ -2384,34 +2384,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C14" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="I14" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="D14" s="7" t="n">
-        <v>58</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>76</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>65</v>
-      </c>
-      <c r="G14" s="8" t="n">
-        <v>85</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>38</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>50</v>
-      </c>
       <c r="J14" s="7" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
@@ -2424,7 +2424,7 @@
         <v>229</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17">
@@ -2434,10 +2434,10 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="19">
@@ -2454,10 +2454,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C20" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="21">
@@ -2470,7 +2470,7 @@
         <v>229</v>
       </c>
       <c r="C21" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -2591,28 +2591,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="D5" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="E5" t="n">
-        <v>1057.61</v>
+        <v>1057.02</v>
       </c>
       <c r="F5" t="n">
-        <v>1215.64</v>
+        <v>1215.54</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1057.61</v>
+        <v>1057.02</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1215.64</v>
+        <v>1215.54</v>
       </c>
       <c r="I5" s="22" t="n">
-        <v>121.918</v>
+        <v>121.872</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>140.144</v>
+        <v>140.154</v>
       </c>
     </row>
     <row r="6">
@@ -2630,25 +2630,25 @@
         <v>229</v>
       </c>
       <c r="D6" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E6" t="n">
-        <v>354.75</v>
+        <v>355.37</v>
       </c>
       <c r="F6" t="n">
-        <v>461.36</v>
+        <v>461.03</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>354.75</v>
+        <v>355.37</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>461.36</v>
+        <v>461.03</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>40.914</v>
+        <v>40.958</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>53.175</v>
+        <v>53.165</v>
       </c>
     </row>
     <row r="7">
@@ -2658,25 +2658,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="D7" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="E7" t="n">
-        <v>1412.36</v>
+        <v>1412.39</v>
       </c>
       <c r="F7" t="n">
-        <v>1677</v>
+        <v>1676.57</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>1412.36</v>
+        <v>1412.39</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1677</v>
+        <v>1676.57</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>162.832</v>
+        <v>162.83</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>193.319</v>
@@ -2748,31 +2748,31 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D11" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E11" t="n">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="F11" t="n">
         <v>89</v>
       </c>
       <c r="G11" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="H11" t="n">
-        <v>1215.64</v>
+        <v>1215.54</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>1215.64</v>
+        <v>1215.54</v>
       </c>
       <c r="J11" t="n">
-        <v>140.144</v>
+        <v>140.154</v>
       </c>
     </row>
     <row r="12">
@@ -2782,31 +2782,31 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>45</v>
+      </c>
+      <c r="C12" t="n">
+        <v>78</v>
+      </c>
+      <c r="D12" t="n">
+        <v>86</v>
+      </c>
+      <c r="E12" t="n">
         <v>54</v>
       </c>
-      <c r="C12" t="n">
-        <v>76</v>
-      </c>
-      <c r="D12" t="n">
-        <v>85</v>
-      </c>
-      <c r="E12" t="n">
-        <v>50</v>
-      </c>
       <c r="F12" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G12" t="n">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="H12" t="n">
-        <v>461.36</v>
+        <v>461.03</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>461.36</v>
+        <v>461.03</v>
       </c>
       <c r="J12" t="n">
-        <v>53.175</v>
+        <v>53.165</v>
       </c>
     </row>
     <row r="14">
@@ -2906,10 +2906,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>651.16</v>
+        <v>651.29</v>
       </c>
       <c r="C20" t="n">
-        <v>773.28</v>
+        <v>773</v>
       </c>
     </row>
     <row r="21">
@@ -2919,10 +2919,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="C21" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
   </sheetData>
@@ -3060,10 +3060,10 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="23" t="n">
         <v>15</v>
-      </c>
-      <c r="C5" s="23" t="n">
-        <v>18</v>
       </c>
       <c r="D5" s="22" t="n">
         <v>22</v>
@@ -3072,22 +3072,22 @@
         <v>26</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G5" s="23" t="n">
         <v>29</v>
       </c>
       <c r="H5" s="22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="22" t="n">
         <v>10</v>
       </c>
       <c r="K5" s="23" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -3097,28 +3097,28 @@
         </is>
       </c>
       <c r="B6" s="22" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" s="23" t="n">
         <v>37</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="D6" s="22" t="n">
+        <v>54</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>64</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>60</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>71</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>38</v>
+      </c>
+      <c r="I6" s="23" t="n">
         <v>44</v>
-      </c>
-      <c r="D6" s="22" t="n">
-        <v>53</v>
-      </c>
-      <c r="E6" s="23" t="n">
-        <v>62</v>
-      </c>
-      <c r="F6" s="22" t="n">
-        <v>59</v>
-      </c>
-      <c r="G6" s="23" t="n">
-        <v>69</v>
-      </c>
-      <c r="H6" s="22" t="n">
-        <v>34</v>
-      </c>
-      <c r="I6" s="23" t="n">
-        <v>40</v>
       </c>
       <c r="J6" s="22" t="n">
         <v>23</v>
@@ -3134,10 +3134,10 @@
         </is>
       </c>
       <c r="B7" s="22" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" s="23" t="n">
         <v>22</v>
-      </c>
-      <c r="C7" s="23" t="n">
-        <v>26</v>
       </c>
       <c r="D7" s="22" t="n">
         <v>32</v>
@@ -3146,22 +3146,22 @@
         <v>38</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J7" s="22" t="n">
         <v>14</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -3171,10 +3171,10 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" s="23" t="n">
         <v>18</v>
-      </c>
-      <c r="C8" s="23" t="n">
-        <v>22</v>
       </c>
       <c r="D8" s="22" t="n">
         <v>26</v>
@@ -3186,16 +3186,16 @@
         <v>29</v>
       </c>
       <c r="G8" s="23" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K8" s="23" t="n">
         <v>14</v>
@@ -3245,10 +3245,10 @@
         </is>
       </c>
       <c r="B10" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" s="23" t="n">
         <v>19</v>
-      </c>
-      <c r="C10" s="23" t="n">
-        <v>22</v>
       </c>
       <c r="D10" s="22" t="n">
         <v>27</v>
@@ -3260,16 +3260,16 @@
         <v>30</v>
       </c>
       <c r="G10" s="23" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J10" s="22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K10" s="23" t="n">
         <v>14</v>
@@ -3282,34 +3282,34 @@
         </is>
       </c>
       <c r="B11" s="22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C11" s="23" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D11" s="22" t="n">
         <v>22</v>
       </c>
       <c r="E11" s="23" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F11" s="22" t="n">
         <v>25</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J11" s="22" t="n">
         <v>10</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -3319,28 +3319,28 @@
         </is>
       </c>
       <c r="B12" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="23" t="n">
         <v>13</v>
-      </c>
-      <c r="C12" s="23" t="n">
-        <v>16</v>
       </c>
       <c r="D12" s="22" t="n">
         <v>19</v>
       </c>
       <c r="E12" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="F12" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="F12" s="22" t="n">
-        <v>21</v>
-      </c>
       <c r="G12" s="23" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I12" s="23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J12" s="22" t="n">
         <v>9</v>
@@ -3356,28 +3356,28 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="C13" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="C13" s="23" t="n">
-        <v>28</v>
-      </c>
       <c r="D13" s="22" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E13" s="23" t="n">
         <v>40</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G13" s="23" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I13" s="23" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J13" s="22" t="n">
         <v>15</v>
@@ -3393,34 +3393,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>163</v>
+        <v>138</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>195</v>
+        <v>164</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>180</v>
+        <v>197</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16">
@@ -3478,7 +3478,7 @@
         <v>206</v>
       </c>
       <c r="C19" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D19" t="n">
         <v>10.7</v>
@@ -3491,10 +3491,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C20" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D20" t="n">
         <v>6.4</v>
@@ -3507,10 +3507,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C21" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D21" t="n">
         <v>5.3</v>
@@ -3558,7 +3558,7 @@
         <v>86</v>
       </c>
       <c r="C24" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D24" t="n">
         <v>4.5</v>
@@ -3590,7 +3590,7 @@
         <v>131</v>
       </c>
       <c r="C26" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D26" t="n">
         <v>6.8</v>
@@ -3680,10 +3680,10 @@
         <v>67</v>
       </c>
       <c r="C6" t="n">
+        <v>138</v>
+      </c>
+      <c r="D6" t="n">
         <v>164</v>
-      </c>
-      <c r="D6" t="n">
-        <v>195</v>
       </c>
     </row>
     <row r="7">
@@ -3696,10 +3696,10 @@
         <v>69</v>
       </c>
       <c r="C7" t="n">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D7" t="n">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8">
@@ -3712,10 +3712,10 @@
         <v>72</v>
       </c>
       <c r="C8" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D8" t="n">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9">
@@ -3728,10 +3728,10 @@
         <v>75</v>
       </c>
       <c r="C9" t="n">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="D9" t="n">
-        <v>180</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10">
@@ -3758,10 +3758,10 @@
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>651.16</v>
+        <v>651.29</v>
       </c>
       <c r="D12" t="n">
-        <v>773.28</v>
+        <v>773</v>
       </c>
     </row>
     <row r="14">
@@ -3800,7 +3800,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="18">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>912 – 1083 und</t>
+          <t>910 – 1080 und</t>
         </is>
       </c>
     </row>
@@ -4097,21 +4097,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Ajustada: M 25% · S 22% · XS 18.0% (recibe lo restado de M y S).</t>
+          <t xml:space="preserve">   Ajustada: M 25% · S 22% · XS 15.2% (recibe lo restado de M y S).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 16.6% · XL 11.3%.</t>
+          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 18.2% · XL 11.3%.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">   XS objetivo 18%: exceso de XS repartido por igual a S y M (criterio I+D).</t>
+          <t xml:space="preserve">   XS objetivo 15.2%: +1.6 pp a L; excedente repartido entre S y M.</t>
         </is>
       </c>
     </row>

</xml_diff>